<commit_message>
Phase 3 on Zoho Inventory behind the rehearsal switch (0065): stock master ctp|zoho, Zoho physical-stock cache on parts, Ship in Zoho (package+shipment, record_goods_out), count -> Inventory adjustment, purchase receives, webhooks (hook, refetch-only); live-tested on TEST docs; inv_fixture/inv_get; webhook setup doc; dry run refreshed; SW v29
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cutover/dryrun_2026-10-23.xlsx
+++ b/docs/cutover/dryrun_2026-10-23.xlsx
@@ -440,7 +440,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Zoho read at 2026-10-23T10:35:58.918Z</t>
+          <t>Zoho read at 2026-10-23T11:14:45.763Z</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>{"packages": "not readable (401 You are not authorized to perform this operation)", "shipmentorders": "not readable (401 You are not authorized to perform this operation)", "purchasereceives": "not readable (401 You are not authorized to perform this operation)", "inventoryadjustments": "not readable (401 You are not authorized to perform this operation)", "transferorders": "not readable (401 You are not authorized to perform this operation)"}</t>
+          <t>{"packages": "3 found", "shipmentorders": "3 found", "purchasereceives": "0 found", "inventoryadjustments": "0 found", "transferorders": "0 found"}</t>
         </is>
       </c>
     </row>

</xml_diff>